<commit_message>
FA: reporte manual relee DBF y reconcilia con SQL (compara DBF vs SQL); H_Tiendas auto-cura con Id IDENTITY; RegistrosDBF real en FA; log de errores al leer FC*.DBF
</commit_message>
<xml_diff>
--- a/Ventas_Mensuales_JULIO_2026.xlsx
+++ b/Ventas_Mensuales_JULIO_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>JULIO (2026)</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t>06:00 AM</t>
+  </si>
+  <si>
+    <t>05:00 PM</t>
   </si>
   <si>
     <t>03:00 AM</t>
@@ -594,10 +597,10 @@
         <v>11</v>
       </c>
       <c r="C5" s="4">
-        <v>24.456922344700303</v>
+        <v>24.36395512678552</v>
       </c>
       <c r="D5" s="5">
-        <v>137621</v>
+        <v>72248</v>
       </c>
       <c r="E5" s="5" t="str">
         <f>=D5/31</f>
@@ -606,16 +609,16 @@
         <v>12</v>
       </c>
       <c r="G5" s="5">
-        <v>12754</v>
+        <v>6759</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I5" s="5">
-        <v>420</v>
+        <v>216</v>
       </c>
       <c r="J5" s="6">
-        <v>3365786.1100000003</v>
+        <v>1760247.0300000003</v>
       </c>
       <c r="K5" s="6" t="str">
         <f>=J5/31</f>
@@ -626,10 +629,10 @@
         <v>11</v>
       </c>
       <c r="C6" s="4">
-        <v>22.033022536937427</v>
+        <v>21.918779251170047</v>
       </c>
       <c r="D6" s="5">
-        <v>73435</v>
+        <v>38460</v>
       </c>
       <c r="E6" s="5" t="str">
         <f>=D6/31</f>
@@ -638,16 +641,16 @@
         <v>12</v>
       </c>
       <c r="G6" s="5">
-        <v>8164</v>
+        <v>4251</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>14</v>
       </c>
       <c r="I6" s="5">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="J6" s="6">
-        <v>1617995.01</v>
+        <v>842996.25</v>
       </c>
       <c r="K6" s="6" t="str">
         <f>=J6/31</f>
@@ -658,10 +661,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="4">
-        <v>29.060145528280216</v>
+        <v>29.021990931645142</v>
       </c>
       <c r="D7" s="5">
-        <v>55728</v>
+        <v>58445</v>
       </c>
       <c r="E7" s="5" t="str">
         <f>=D7/31</f>
@@ -670,16 +673,16 @@
         <v>15</v>
       </c>
       <c r="G7" s="5">
-        <v>4140</v>
+        <v>4288</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>16</v>
       </c>
       <c r="I7" s="5">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J7" s="6">
-        <v>1619463.7899999998</v>
+        <v>1696190.2600000002</v>
       </c>
       <c r="K7" s="6" t="str">
         <f>=J7/31</f>
@@ -690,10 +693,10 @@
         <v>11</v>
       </c>
       <c r="C8" s="4">
-        <v>33.01108255187738</v>
+        <v>32.840328371592534</v>
       </c>
       <c r="D8" s="5">
-        <v>53106</v>
+        <v>55760</v>
       </c>
       <c r="E8" s="5" t="str">
         <f>=D8/31</f>
@@ -702,16 +705,16 @@
         <v>17</v>
       </c>
       <c r="G8" s="5">
-        <v>3929</v>
+        <v>4069</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>16</v>
       </c>
       <c r="I8" s="5">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="J8" s="6">
-        <v>1753086.55</v>
+        <v>1831176.7099999997</v>
       </c>
       <c r="K8" s="6" t="str">
         <f>=J8/31</f>
@@ -722,10 +725,10 @@
         <v>11</v>
       </c>
       <c r="C9" s="4">
-        <v>31.432541214705356</v>
+        <v>31.312218034135856</v>
       </c>
       <c r="D9" s="5">
-        <v>72001</v>
+        <v>75346</v>
       </c>
       <c r="E9" s="5" t="str">
         <f>=D9/31</f>
@@ -734,16 +737,16 @@
         <v>15</v>
       </c>
       <c r="G9" s="5">
-        <v>5202</v>
+        <v>5372</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>16</v>
       </c>
       <c r="I9" s="5">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="J9" s="6">
-        <v>2263174.4000000004</v>
+        <v>2359250.3800000004</v>
       </c>
       <c r="K9" s="6" t="str">
         <f>=J9/31</f>
@@ -754,10 +757,10 @@
         <v>11</v>
       </c>
       <c r="C10" s="4">
-        <v>26.196709465278325</v>
+        <v>26.061759164906178</v>
       </c>
       <c r="D10" s="5">
-        <v>38319</v>
+        <v>40235</v>
       </c>
       <c r="E10" s="5" t="str">
         <f>=D10/31</f>
@@ -766,7 +769,7 @@
         <v>18</v>
       </c>
       <c r="G10" s="5">
-        <v>3328</v>
+        <v>3522</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>19</v>
@@ -775,7 +778,7 @@
         <v>1</v>
       </c>
       <c r="J10" s="6">
-        <v>1003831.7100000001</v>
+        <v>1048594.8800000001</v>
       </c>
       <c r="K10" s="6" t="str">
         <f>=J10/31</f>
@@ -786,28 +789,28 @@
         <v>11</v>
       </c>
       <c r="C11" s="4">
-        <v>27.949559588168455</v>
+        <v>27.90985052855855</v>
       </c>
       <c r="D11" s="5">
-        <v>58082</v>
+        <v>61015</v>
       </c>
       <c r="E11" s="5" t="str">
         <f>=D11/31</f>
       </c>
       <c r="F11" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G11" s="5">
-        <v>4389</v>
+        <v>4561</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>16</v>
       </c>
       <c r="I11" s="5">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="J11" s="6">
-        <v>1623366.3200000003</v>
+        <v>1702919.53</v>
       </c>
       <c r="K11" s="6" t="str">
         <f>=J11/31</f>
@@ -818,10 +821,10 @@
         <v>11</v>
       </c>
       <c r="C12" s="4">
-        <v>24.819793730061967</v>
+        <v>24.798692671884716</v>
       </c>
       <c r="D12" s="5">
-        <v>59873</v>
+        <v>62731</v>
       </c>
       <c r="E12" s="5" t="str">
         <f>=D12/31</f>
@@ -830,16 +833,16 @@
         <v>12</v>
       </c>
       <c r="G12" s="5">
-        <v>4396</v>
+        <v>4730</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>16</v>
       </c>
       <c r="I12" s="5">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="J12" s="6">
-        <v>1486035.5100000002</v>
+        <v>1555646.79</v>
       </c>
       <c r="K12" s="6" t="str">
         <f>=J12/31</f>
@@ -850,28 +853,28 @@
         <v>11</v>
       </c>
       <c r="C13" s="4">
-        <v>30.54827943909444</v>
+        <v>30.360764750093953</v>
       </c>
       <c r="D13" s="5">
-        <v>29595</v>
+        <v>31932</v>
       </c>
       <c r="E13" s="5" t="str">
         <f>=D13/31</f>
       </c>
       <c r="F13" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G13" s="5">
-        <v>2579</v>
+        <v>2748</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I13" s="5">
         <v>0</v>
       </c>
       <c r="J13" s="6">
-        <v>904076.33</v>
+        <v>969479.9400000001</v>
       </c>
       <c r="K13" s="6" t="str">
         <f>=J13/31</f>
@@ -879,22 +882,22 @@
     </row>
     <row r="14" ht="15" customHeight="true">
       <c r="B14" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" s="8">
-        <v>19.024600042890842</v>
+        <v>18.911774686121483</v>
       </c>
       <c r="D14" s="9">
-        <v>27978</v>
+        <v>29470</v>
       </c>
       <c r="E14" s="9" t="str">
         <f>=D14/31</f>
       </c>
       <c r="F14" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" s="9">
-        <v>3332</v>
+        <v>3537</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>16</v>
@@ -903,7 +906,7 @@
         <v>34</v>
       </c>
       <c r="J14" s="10">
-        <v>532270.26</v>
+        <v>557330.0000000001</v>
       </c>
       <c r="K14" s="10" t="str">
         <f>=J14/31</f>
@@ -911,13 +914,13 @@
     </row>
     <row r="15" ht="15" customHeight="true">
       <c r="B15" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="8">
-        <v>20.040157551204143</v>
+        <v>20.23284280100036</v>
       </c>
       <c r="D15" s="9">
-        <v>26658</v>
+        <v>27990</v>
       </c>
       <c r="E15" s="9" t="str">
         <f>=D15/31</f>
@@ -926,16 +929,16 @@
         <v>17</v>
       </c>
       <c r="G15" s="9">
-        <v>2277</v>
+        <v>2343</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>13</v>
       </c>
       <c r="I15" s="9">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J15" s="10">
-        <v>534230.52</v>
+        <v>566317.27</v>
       </c>
       <c r="K15" s="10" t="str">
         <f>=J15/31</f>
@@ -943,13 +946,13 @@
     </row>
     <row r="16" ht="15" customHeight="true">
       <c r="B16" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" s="8">
-        <v>25.069880623187426</v>
+        <v>24.940576310454677</v>
       </c>
       <c r="D16" s="9">
-        <v>29654</v>
+        <v>31077</v>
       </c>
       <c r="E16" s="9" t="str">
         <f>=D16/31</f>
@@ -958,16 +961,16 @@
         <v>15</v>
       </c>
       <c r="G16" s="9">
-        <v>2321</v>
+        <v>2405</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I16" s="9">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J16" s="10">
-        <v>743422.24</v>
+        <v>775078.29</v>
       </c>
       <c r="K16" s="10" t="str">
         <f>=J16/31</f>
@@ -975,13 +978,13 @@
     </row>
     <row r="17" ht="15" customHeight="true">
       <c r="B17" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C17" s="8">
-        <v>20.815476450024434</v>
+        <v>20.716651412227385</v>
       </c>
       <c r="D17" s="9">
-        <v>26603</v>
+        <v>27970</v>
       </c>
       <c r="E17" s="9" t="str">
         <f>=D17/31</f>
@@ -990,7 +993,7 @@
         <v>17</v>
       </c>
       <c r="G17" s="9">
-        <v>2340</v>
+        <v>2400</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>19</v>
@@ -999,7 +1002,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="10">
-        <v>553754.12</v>
+        <v>579444.74</v>
       </c>
       <c r="K17" s="10" t="str">
         <f>=J17/31</f>
@@ -1007,22 +1010,22 @@
     </row>
     <row r="18" ht="15" customHeight="true">
       <c r="B18" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="8">
-        <v>19.75450026521179</v>
+        <v>19.752641700039685</v>
       </c>
       <c r="D18" s="9">
-        <v>26394</v>
+        <v>27717</v>
       </c>
       <c r="E18" s="9" t="str">
         <f>=D18/31</f>
       </c>
       <c r="F18" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G18" s="9">
-        <v>2407</v>
+        <v>2520</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>19</v>
@@ -1031,7 +1034,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="10">
-        <v>521400.2799999999</v>
+        <v>547483.97</v>
       </c>
       <c r="K18" s="10" t="str">
         <f>=J18/31</f>
@@ -1039,13 +1042,13 @@
     </row>
     <row r="19" ht="15" customHeight="true">
       <c r="B19" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="8">
-        <v>24.2910843198137</v>
+        <v>24.228764372469637</v>
       </c>
       <c r="D19" s="9">
-        <v>41224</v>
+        <v>43225</v>
       </c>
       <c r="E19" s="9" t="str">
         <f>=D19/31</f>
@@ -1054,16 +1057,16 @@
         <v>15</v>
       </c>
       <c r="G19" s="9">
-        <v>3273</v>
+        <v>3389</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I19" s="9">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J19" s="10">
-        <v>1001375.6599999999</v>
+        <v>1047288.3400000001</v>
       </c>
       <c r="K19" s="10" t="str">
         <f>=J19/31</f>
@@ -1071,13 +1074,13 @@
     </row>
     <row r="20" ht="15" customHeight="true">
       <c r="B20" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C20" s="12">
-        <v>30.307250623441398</v>
+        <v>29.971442873969373</v>
       </c>
       <c r="D20" s="13">
-        <v>1604</v>
+        <v>1698</v>
       </c>
       <c r="E20" s="13" t="str">
         <f>=D20/31</f>
@@ -1086,16 +1089,16 @@
         <v>12</v>
       </c>
       <c r="G20" s="13">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I20" s="13">
         <v>1</v>
       </c>
       <c r="J20" s="14">
-        <v>48612.83</v>
+        <v>50891.509999999995</v>
       </c>
       <c r="K20" s="14" t="str">
         <f>=J20/31</f>
@@ -1103,13 +1106,13 @@
     </row>
     <row r="21" ht="15" customHeight="true">
       <c r="B21" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C21" s="12">
-        <v>33.17385790031813</v>
+        <v>32.4581473941368</v>
       </c>
       <c r="D21" s="13">
-        <v>4715</v>
+        <v>4912</v>
       </c>
       <c r="E21" s="13" t="str">
         <f>=D21/31</f>
@@ -1118,16 +1121,16 @@
         <v>17</v>
       </c>
       <c r="G21" s="13">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I21" s="13">
         <v>8</v>
       </c>
       <c r="J21" s="14">
-        <v>156414.74</v>
+        <v>159434.41999999998</v>
       </c>
       <c r="K21" s="14" t="str">
         <f>=J21/31</f>
@@ -1135,13 +1138,13 @@
     </row>
     <row r="22" ht="15" customHeight="true">
       <c r="B22" s="15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C22" s="16">
-        <v>13.530474137931037</v>
+        <v>13.542379912663753</v>
       </c>
       <c r="D22" s="17">
-        <v>11832</v>
+        <v>12366</v>
       </c>
       <c r="E22" s="17" t="str">
         <f>=D22/31</f>
@@ -1150,16 +1153,16 @@
         <v>15</v>
       </c>
       <c r="G22" s="17">
-        <v>1259</v>
+        <v>1300</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>13</v>
       </c>
       <c r="I22" s="17">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J22" s="18">
-        <v>160092.57000000004</v>
+        <v>167465.06999999998</v>
       </c>
       <c r="K22" s="18" t="str">
         <f>=J22/31</f>
@@ -1167,13 +1170,13 @@
     </row>
     <row r="23" ht="15" customHeight="true">
       <c r="B23" s="15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C23" s="16">
-        <v>14.329568666890154</v>
+        <v>14.356858906150245</v>
       </c>
       <c r="D23" s="17">
-        <v>8949</v>
+        <v>9398</v>
       </c>
       <c r="E23" s="17" t="str">
         <f>=D23/31</f>
@@ -1182,16 +1185,16 @@
         <v>15</v>
       </c>
       <c r="G23" s="17">
-        <v>979</v>
+        <v>1021</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I23" s="17">
         <v>12</v>
       </c>
       <c r="J23" s="18">
-        <v>128235.30999999998</v>
+        <v>134925.76</v>
       </c>
       <c r="K23" s="18" t="str">
         <f>=J23/31</f>

</xml_diff>